<commit_message>
Switching to external participant identifiers
</commit_message>
<xml_diff>
--- a/analysis/ExperimentLogExample.xlsx
+++ b/analysis/ExperimentLogExample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories\SensorySurvey3D\analysis\private_utils\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories\SensorySurvey3D\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8414C8AC-B880-4050-8A29-CA62DB9188A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F96C3B-07C1-42F0-B66B-C8D71D6FE210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2130" yWindow="1965" windowWidth="37290" windowHeight="20565" xr2:uid="{276D3F31-1118-48AD-A056-B5311D6F72EF}"/>
+    <workbookView xWindow="165" yWindow="675" windowWidth="21315" windowHeight="11835" xr2:uid="{276D3F31-1118-48AD-A056-B5311D6F72EF}"/>
   </bookViews>
   <sheets>
     <sheet name="ExperimentLog" sheetId="1" r:id="rId1"/>
@@ -37,18 +37,12 @@
     <t>Survey3D</t>
   </si>
   <si>
-    <t>S113</t>
-  </si>
-  <si>
     <t>Electrodes</t>
   </si>
   <si>
     <t>1,1,1,1,1,1,1,1,1,9,9,9,9,9,9,9,9,9,9</t>
   </si>
   <si>
-    <t>Pro1</t>
-  </si>
-  <si>
     <t>1:19</t>
   </si>
   <si>
@@ -83,6 +77,12 @@
   </si>
   <si>
     <t>251113_0000</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>R2</t>
   </si>
 </sst>
 </file>
@@ -990,16 +990,16 @@
         <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1007,22 +1007,22 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H2" s="7">
         <v>45971</v>
@@ -1033,22 +1033,22 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H3" s="7">
         <v>45974</v>

</xml_diff>